<commit_message>
fix: optimize processing pipeline, enhance OCR and alert tracking, and update dashboard UI
</commit_message>
<xml_diff>
--- a/data/detections.xlsx
+++ b/data/detections.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detected Vehicles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detected Vehicles" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,53 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00856404"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD2D2"/>
+        <bgColor rgb="00FFD2D2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +86,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,43 +465,316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Vehicle Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Plate Number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Confidence (%)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>First Seen (Video Time)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DB4E59</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>00:10</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:20:39</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Missing Number Plate</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>00:08</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:20:41</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Missing Plate</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Q8C5E1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>00:18</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:20:45</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>5392E02</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>00:22</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:20:49</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Missing Number Plate</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>00:18</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:21:18</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Missing Plate</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Truck</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Missing Number Plate</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>00:21</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:21:18</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Missing Plate</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Missing Number Plate</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>00:52</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:21:18</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Missing Plate</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Bike</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>TN 50A P8219</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>00:01</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:21:18</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>FLAGGED (RED)</t>
         </is>
       </c>
     </row>

</xml_diff>